<commit_message>
Update soccer trades 2026-08-06 22:02:23 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Jupiler League/trades.xlsx
+++ b/data/sxbet/ligas/Jupiler League/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,28 +531,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xae1c40433a387d3e160c3f482c36c347908d7b62a6d9acbef1b9a3417e77039c</t>
+          <t>0x8e5a34b35110bb5418a07b52d7e0f879e10398e7e68e1c0e54ba1d17927f58bc</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>18.15</t>
+          <t>2.62</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.2275</t>
+          <t>1.3237</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -578,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xb7e709d4c259327ee20c2eac233626397889f1c291812b5ccb8dd8c68a28d3ba</t>
+          <t>0x4937d8af628761601484db1ccd581e7d2dde4744b925fb09c660b5030bd65ec9</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786047040</t>
+          <t>1786053446</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>79.78022</t>
+          <t>8.092664</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,110 +635,214 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>0xae1c40433a387d3e160c3f482c36c347908d7b62a6d9acbef1b9a3417e77039c</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>18.15</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.2275</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Jupiler League</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Club Brugge KV vs KV Kortrijk</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Club Brugge KV</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>KV Kortrijk</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0xb7e709d4c259327ee20c2eac233626397889f1c291812b5ccb8dd8c68a28d3ba</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19453184</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>1786047040</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1786128300</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>79.78022</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>0x17da446efa49f610050e7ecaeaec91964befc8f9d839eaf4eaf250bb1dc857a8</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>0.00029</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>1.15</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Jupiler League</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Club Brugge KV vs KV Kortrijk</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Club Brugge KV</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>KV Kortrijk</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>0xd77ddb73d8a9ad095981816a0ffa614e557d5ed0af33c43936807c64f20a7c18</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>L19453184</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>1786046726</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>1786128300</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>0.001933</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-07 03:02:59 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Jupiler League/trades.xlsx
+++ b/data/sxbet/ligas/Jupiler League/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x8e5a34b35110bb5418a07b52d7e0f879e10398e7e68e1c0e54ba1d17927f58bc</t>
+          <t>0x9df37bdd2a6c3b8b897002cd51096c135c9168d7b8947a1d6316f2f8dae3e828</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -542,17 +542,17 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.62</t>
+          <t>2.06637</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.3237</t>
+          <t>1.1713</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -578,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x4937d8af628761601484db1ccd581e7d2dde4744b925fb09c660b5030bd65ec9</t>
+          <t>0xe2658f37be5ea92097979a1992f5c8cce5e7389795f21ff51094a41bf3c0231c</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786053446</t>
+          <t>1786068821</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>8.092664</t>
+          <t>12.066394</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,28 +635,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xae1c40433a387d3e160c3f482c36c347908d7b62a6d9acbef1b9a3417e77039c</t>
+          <t>0x8e5a34b35110bb5418a07b52d7e0f879e10398e7e68e1c0e54ba1d17927f58bc</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>18.15</t>
+          <t>2.62</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.2275</t>
+          <t>1.3237</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -682,7 +682,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xb7e709d4c259327ee20c2eac233626397889f1c291812b5ccb8dd8c68a28d3ba</t>
+          <t>0x4937d8af628761601484db1ccd581e7d2dde4744b925fb09c660b5030bd65ec9</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786047040</t>
+          <t>1786053446</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>79.78022</t>
+          <t>8.092664</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,110 +739,214 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>0xae1c40433a387d3e160c3f482c36c347908d7b62a6d9acbef1b9a3417e77039c</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>18.15</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.2275</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Jupiler League</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Club Brugge KV vs KV Kortrijk</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Club Brugge KV</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>KV Kortrijk</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0xb7e709d4c259327ee20c2eac233626397889f1c291812b5ccb8dd8c68a28d3ba</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19453184</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1786047040</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1786128300</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>79.78022</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>0x17da446efa49f610050e7ecaeaec91964befc8f9d839eaf4eaf250bb1dc857a8</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>0.00029</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>1.15</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Jupiler League</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Club Brugge KV vs KV Kortrijk</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Club Brugge KV</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>KV Kortrijk</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>0xd77ddb73d8a9ad095981816a0ffa614e557d5ed0af33c43936807c64f20a7c18</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>L19453184</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>1786046726</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>1786128300</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>0.001933</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>